<commit_message>
Realizado a parte de emprestimo de viaturas
</commit_message>
<xml_diff>
--- a/data/qff_cmm.xlsx
+++ b/data/qff_cmm.xlsx
@@ -1,19 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="153222"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\frotinha\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="7635"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="296">
   <si>
     <t>805002000</t>
   </si>
@@ -466,9 +472,6 @@
   </si>
   <si>
     <t>DF/CIAP</t>
-  </si>
-  <si>
-    <t>303020000</t>
   </si>
   <si>
     <t>Sede</t>
@@ -909,15 +912,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="9"/>
       <color rgb="FF000000"/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -937,293 +940,613 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
-    <border/>
-    <border/>
-    <border/>
-    <border/>
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+  <a:themeElements>
+    <a:clrScheme name="Escritório">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4472C4"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Escritório">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Escritório">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AW73"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:49">
       <c r="G1" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+      <c r="U1" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="W1" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="X1" s="9"/>
+      <c r="Y1" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
+      <c r="AB1" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="AE1" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
+      <c r="AJ1" s="9"/>
+      <c r="AK1" s="9"/>
+      <c r="AL1" s="9"/>
+      <c r="AM1" s="9"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="9"/>
+      <c r="AP1" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="AQ1" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="AR1" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="AS1" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="AT1" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="AU1" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="AV1" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="AW1" s="9" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="2" spans="1:49" ht="138.75">
+      <c r="A2" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K2" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5" t="s">
+      <c r="N2" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O2" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P2" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q2" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="R2" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5" t="s">
+      <c r="S2" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="U2" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5" t="s">
+      <c r="V2" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W2" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="X2" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="Y2" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5" t="s">
+      <c r="Z2" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA2" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="AB2" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="Z1" s="5"/>
-      <c r="AA1" s="5"/>
-      <c r="AB1" s="5" t="s">
+      <c r="AC2" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD2" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AE2" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AF2" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="AG2" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="AH2" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="AJ2" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="AK2" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="AL2" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="AM2" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="AN2" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="AO2" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="AP2" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="AF1" s="5"/>
-      <c r="AG1" s="5"/>
-      <c r="AH1" s="5"/>
-      <c r="AI1" s="5"/>
-      <c r="AJ1" s="5"/>
-      <c r="AK1" s="5"/>
-      <c r="AL1" s="5"/>
-      <c r="AM1" s="5"/>
-      <c r="AN1" s="5"/>
-      <c r="AO1" s="5"/>
-      <c r="AP1" s="5" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="AQ1" s="5" t="s">
+      <c r="AR2" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="AR1" s="5" t="s">
+      <c r="AS2" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="AS1" s="5" t="s">
+      <c r="AT2" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="AT1" s="5" t="s">
+      <c r="AU2" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AV2" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="AV1" s="5" t="s">
+      <c r="AW2" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="AW1" s="5" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>292</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="V2" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="X2" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="Y2" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="Z2" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="AA2" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="AB2" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="AC2" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="AD2" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="AE2" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="AF2" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="AG2" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="AH2" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="AI2" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="AJ2" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="AK2" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="AL2" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="AM2" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="AN2" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="AO2" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="AP2" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="AQ2" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="AR2" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="AS2" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="AT2" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="AU2" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="AV2" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="AW2" s="5" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" spans="1:49">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1294,7 +1617,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:49">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -1365,7 +1688,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:49">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1436,7 +1759,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:49">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1507,7 +1830,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:49">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1578,7 +1901,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:49">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1649,7 +1972,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:49">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -1720,7 +2043,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:49">
       <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
@@ -1791,7 +2114,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:49">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
@@ -1862,12 +2185,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="B12" s="3" t="s">
+    <row r="12" spans="1:49">
+      <c r="A12" s="8" t="s">
         <v>215</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>214</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>38</v>
@@ -1929,9 +2252,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
+    <row r="13" spans="1:49">
+      <c r="A13" s="8"/>
+      <c r="B13" s="7"/>
       <c r="C13" s="1" t="s">
         <v>41</v>
       </c>
@@ -1992,9 +2315,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2"/>
-      <c r="B14" s="3"/>
+    <row r="14" spans="1:49">
+      <c r="A14" s="8"/>
+      <c r="B14" s="7"/>
       <c r="C14" s="1" t="s">
         <v>44</v>
       </c>
@@ -2055,9 +2378,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
+    <row r="15" spans="1:49">
+      <c r="A15" s="8"/>
+      <c r="B15" s="7"/>
       <c r="C15" s="1" t="s">
         <v>47</v>
       </c>
@@ -2118,9 +2441,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2"/>
-      <c r="B16" s="3"/>
+    <row r="16" spans="1:49">
+      <c r="A16" s="8"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="1" t="s">
         <v>50</v>
       </c>
@@ -2185,9 +2508,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2"/>
-      <c r="B17" s="3"/>
+    <row r="17" spans="1:49">
+      <c r="A17" s="8"/>
+      <c r="B17" s="7"/>
       <c r="C17" s="1" t="s">
         <v>53</v>
       </c>
@@ -2248,9 +2571,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2"/>
-      <c r="B18" s="3"/>
+    <row r="18" spans="1:49">
+      <c r="A18" s="8"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="1" t="s">
         <v>56</v>
       </c>
@@ -2313,9 +2636,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2"/>
-      <c r="B19" s="3"/>
+    <row r="19" spans="1:49">
+      <c r="A19" s="8"/>
+      <c r="B19" s="7"/>
       <c r="C19" s="1" t="s">
         <v>59</v>
       </c>
@@ -2376,9 +2699,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2"/>
-      <c r="B20" s="3"/>
+    <row r="20" spans="1:49">
+      <c r="A20" s="8"/>
+      <c r="B20" s="7"/>
       <c r="C20" s="1" t="s">
         <v>62</v>
       </c>
@@ -2441,9 +2764,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2"/>
-      <c r="B21" s="3"/>
+    <row r="21" spans="1:49">
+      <c r="A21" s="8"/>
+      <c r="B21" s="7"/>
       <c r="C21" s="1" t="s">
         <v>65</v>
       </c>
@@ -2506,9 +2829,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2"/>
-      <c r="B22" s="3"/>
+    <row r="22" spans="1:49">
+      <c r="A22" s="8"/>
+      <c r="B22" s="7"/>
       <c r="C22" s="1" t="s">
         <v>68</v>
       </c>
@@ -2569,9 +2892,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2"/>
-      <c r="B23" s="3"/>
+    <row r="23" spans="1:49">
+      <c r="A23" s="8"/>
+      <c r="B23" s="7"/>
       <c r="C23" s="1" t="s">
         <v>71</v>
       </c>
@@ -2632,9 +2955,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2"/>
-      <c r="B24" s="3"/>
+    <row r="24" spans="1:49">
+      <c r="A24" s="8"/>
+      <c r="B24" s="7"/>
       <c r="C24" s="1" t="s">
         <v>74</v>
       </c>
@@ -2699,9 +3022,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="3"/>
+    <row r="25" spans="1:49">
+      <c r="A25" s="8"/>
+      <c r="B25" s="7"/>
       <c r="C25" s="1" t="s">
         <v>77</v>
       </c>
@@ -2762,9 +3085,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="3"/>
+    <row r="26" spans="1:49">
+      <c r="A26" s="8"/>
+      <c r="B26" s="7"/>
       <c r="C26" s="1" t="s">
         <v>80</v>
       </c>
@@ -2837,9 +3160,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2"/>
-      <c r="B27" s="3"/>
+    <row r="27" spans="1:49">
+      <c r="A27" s="8"/>
+      <c r="B27" s="7"/>
       <c r="C27" s="1" t="s">
         <v>83</v>
       </c>
@@ -2900,9 +3223,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
+    <row r="28" spans="1:49">
+      <c r="A28" s="8"/>
+      <c r="B28" s="7"/>
       <c r="C28" s="1" t="s">
         <v>85</v>
       </c>
@@ -2967,9 +3290,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
+    <row r="29" spans="1:49">
+      <c r="A29" s="8"/>
+      <c r="B29" s="7"/>
       <c r="C29" s="1" t="s">
         <v>88</v>
       </c>
@@ -3038,9 +3361,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
+    <row r="30" spans="1:49">
+      <c r="A30" s="8"/>
+      <c r="B30" s="7"/>
       <c r="C30" s="1" t="s">
         <v>91</v>
       </c>
@@ -3103,9 +3426,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2"/>
-      <c r="B31" s="3"/>
+    <row r="31" spans="1:49">
+      <c r="A31" s="8"/>
+      <c r="B31" s="7"/>
       <c r="C31" s="1" t="s">
         <v>93</v>
       </c>
@@ -3184,9 +3507,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2"/>
-      <c r="B32" s="3"/>
+    <row r="32" spans="1:49">
+      <c r="A32" s="8"/>
+      <c r="B32" s="7"/>
       <c r="C32" s="1" t="s">
         <v>96</v>
       </c>
@@ -3247,9 +3570,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2"/>
-      <c r="B33" s="3"/>
+    <row r="33" spans="1:49">
+      <c r="A33" s="8"/>
+      <c r="B33" s="7"/>
       <c r="C33" s="1" t="s">
         <v>99</v>
       </c>
@@ -3314,9 +3637,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2"/>
-      <c r="B34" s="3"/>
+    <row r="34" spans="1:49">
+      <c r="A34" s="8"/>
+      <c r="B34" s="7"/>
       <c r="C34" s="1" t="s">
         <v>102</v>
       </c>
@@ -3377,9 +3700,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2"/>
-      <c r="B35" s="3"/>
+    <row r="35" spans="1:49">
+      <c r="A35" s="8"/>
+      <c r="B35" s="7"/>
       <c r="C35" s="1" t="s">
         <v>105</v>
       </c>
@@ -3440,9 +3763,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2"/>
-      <c r="B36" s="3"/>
+    <row r="36" spans="1:49">
+      <c r="A36" s="8"/>
+      <c r="B36" s="7"/>
       <c r="C36" s="1" t="s">
         <v>108</v>
       </c>
@@ -3505,9 +3828,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2"/>
-      <c r="B37" s="3"/>
+    <row r="37" spans="1:49">
+      <c r="A37" s="8"/>
+      <c r="B37" s="7"/>
       <c r="C37" s="1" t="s">
         <v>111</v>
       </c>
@@ -3580,9 +3903,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2"/>
-      <c r="B38" s="3"/>
+    <row r="38" spans="1:49">
+      <c r="A38" s="8"/>
+      <c r="B38" s="7"/>
       <c r="C38" s="1" t="s">
         <v>114</v>
       </c>
@@ -3651,9 +3974,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2"/>
-      <c r="B39" s="3"/>
+    <row r="39" spans="1:49">
+      <c r="A39" s="8"/>
+      <c r="B39" s="7"/>
       <c r="C39" s="1" t="s">
         <v>117</v>
       </c>
@@ -3724,9 +4047,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2"/>
-      <c r="B40" s="3"/>
+    <row r="40" spans="1:49">
+      <c r="A40" s="8"/>
+      <c r="B40" s="7"/>
       <c r="C40" s="1" t="s">
         <v>120</v>
       </c>
@@ -3795,9 +4118,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2"/>
-      <c r="B41" s="3"/>
+    <row r="41" spans="1:49">
+      <c r="A41" s="8"/>
+      <c r="B41" s="7"/>
       <c r="C41" s="1" t="s">
         <v>123</v>
       </c>
@@ -3878,9 +4201,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2"/>
-      <c r="B42" s="3"/>
+    <row r="42" spans="1:49">
+      <c r="A42" s="8"/>
+      <c r="B42" s="7"/>
       <c r="C42" s="1" t="s">
         <v>126</v>
       </c>
@@ -3949,9 +4272,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2"/>
-      <c r="B43" s="3"/>
+    <row r="43" spans="1:49">
+      <c r="A43" s="8"/>
+      <c r="B43" s="7"/>
       <c r="C43" s="1" t="s">
         <v>129</v>
       </c>
@@ -4022,9 +4345,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2"/>
-      <c r="B44" s="3"/>
+    <row r="44" spans="1:49">
+      <c r="A44" s="8"/>
+      <c r="B44" s="7"/>
       <c r="C44" s="1" t="s">
         <v>132</v>
       </c>
@@ -4099,9 +4422,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2"/>
-      <c r="B45" s="3"/>
+    <row r="45" spans="1:49">
+      <c r="A45" s="8"/>
+      <c r="B45" s="7"/>
       <c r="C45" s="1" t="s">
         <v>135</v>
       </c>
@@ -4182,9 +4505,9 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="2"/>
-      <c r="B46" s="3"/>
+    <row r="46" spans="1:49">
+      <c r="A46" s="8"/>
+      <c r="B46" s="7"/>
       <c r="C46" s="1" t="s">
         <v>138</v>
       </c>
@@ -4265,9 +4588,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2"/>
-      <c r="B47" s="3"/>
+    <row r="47" spans="1:49">
+      <c r="A47" s="8"/>
+      <c r="B47" s="7"/>
       <c r="C47" s="1" t="s">
         <v>141</v>
       </c>
@@ -4330,9 +4653,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2"/>
-      <c r="B48" s="3"/>
+    <row r="48" spans="1:49">
+      <c r="A48" s="8"/>
+      <c r="B48" s="7"/>
       <c r="C48" s="1" t="s">
         <v>144</v>
       </c>
@@ -4401,9 +4724,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2"/>
-      <c r="B49" s="3"/>
+    <row r="49" spans="1:49">
+      <c r="A49" s="8"/>
+      <c r="B49" s="7"/>
       <c r="C49" s="1" t="s">
         <v>147</v>
       </c>
@@ -4466,9 +4789,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2"/>
-      <c r="B50" s="3"/>
+    <row r="50" spans="1:49">
+      <c r="A50" s="8"/>
+      <c r="B50" s="7"/>
       <c r="C50" s="1" t="s">
         <v>150</v>
       </c>
@@ -4535,20 +4858,20 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2"/>
-      <c r="B51" s="3"/>
+    <row r="51" spans="1:49">
+      <c r="A51" s="8"/>
+      <c r="B51" s="7"/>
       <c r="C51" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F51" s="1" t="s">
         <v>151</v>
+      </c>
+      <c r="F51" s="1">
+        <v>201000000</v>
       </c>
       <c r="G51" s="3">
         <v>1</v>
@@ -4606,20 +4929,20 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2"/>
-      <c r="B52" s="3"/>
+    <row r="52" spans="1:49">
+      <c r="A52" s="8"/>
+      <c r="B52" s="7"/>
       <c r="C52" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
@@ -4673,20 +4996,20 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2"/>
-      <c r="B53" s="3"/>
+    <row r="53" spans="1:49">
+      <c r="A53" s="8"/>
+      <c r="B53" s="7"/>
       <c r="C53" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
@@ -4742,20 +5065,20 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2"/>
-      <c r="B54" s="3"/>
+    <row r="54" spans="1:49">
+      <c r="A54" s="8"/>
+      <c r="B54" s="7"/>
       <c r="C54" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
@@ -4819,20 +5142,20 @@
         <v>69</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2"/>
-      <c r="B55" s="3"/>
+    <row r="55" spans="1:49">
+      <c r="A55" s="8"/>
+      <c r="B55" s="7"/>
       <c r="C55" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G55" s="3">
         <v>1</v>
@@ -4888,20 +5211,20 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2"/>
-      <c r="B56" s="3"/>
+    <row r="56" spans="1:49">
+      <c r="A56" s="8"/>
+      <c r="B56" s="7"/>
       <c r="C56" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="3"/>
@@ -4955,20 +5278,20 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2"/>
-      <c r="B57" s="3"/>
+    <row r="57" spans="1:49">
+      <c r="A57" s="8"/>
+      <c r="B57" s="7"/>
       <c r="C57" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
@@ -5030,20 +5353,20 @@
         <v>20</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2"/>
-      <c r="B58" s="3"/>
+    <row r="58" spans="1:49">
+      <c r="A58" s="8"/>
+      <c r="B58" s="7"/>
       <c r="C58" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G58" s="3">
         <v>1</v>
@@ -5099,20 +5422,20 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2"/>
-      <c r="B59" s="3"/>
+    <row r="59" spans="1:49">
+      <c r="A59" s="8"/>
+      <c r="B59" s="7"/>
       <c r="C59" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G59" s="3">
         <v>1</v>
@@ -5170,20 +5493,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2"/>
-      <c r="B60" s="3"/>
+    <row r="60" spans="1:49">
+      <c r="A60" s="8"/>
+      <c r="B60" s="7"/>
       <c r="C60" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
@@ -5243,20 +5566,20 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2"/>
-      <c r="B61" s="3"/>
+    <row r="61" spans="1:49">
+      <c r="A61" s="8"/>
+      <c r="B61" s="7"/>
       <c r="C61" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
@@ -5312,20 +5635,20 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2"/>
-      <c r="B62" s="3"/>
+    <row r="62" spans="1:49">
+      <c r="A62" s="8"/>
+      <c r="B62" s="7"/>
       <c r="C62" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62" s="3"/>
@@ -5379,20 +5702,20 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2"/>
-      <c r="B63" s="3"/>
+    <row r="63" spans="1:49">
+      <c r="A63" s="8"/>
+      <c r="B63" s="7"/>
       <c r="C63" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
@@ -5446,20 +5769,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2"/>
-      <c r="B64" s="3"/>
+    <row r="64" spans="1:49">
+      <c r="A64" s="8"/>
+      <c r="B64" s="7"/>
       <c r="C64" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G64" s="3"/>
       <c r="H64" s="3"/>
@@ -5517,20 +5840,20 @@
         <v>16</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2"/>
-      <c r="B65" s="3"/>
+    <row r="65" spans="1:49">
+      <c r="A65" s="8"/>
+      <c r="B65" s="7"/>
       <c r="C65" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G65" s="3">
         <v>1</v>
@@ -5586,20 +5909,20 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2"/>
-      <c r="B66" s="3"/>
+    <row r="66" spans="1:49">
+      <c r="A66" s="8"/>
+      <c r="B66" s="7"/>
       <c r="C66" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G66" s="3"/>
       <c r="H66" s="3"/>
@@ -5653,20 +5976,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2"/>
-      <c r="B67" s="3"/>
+    <row r="67" spans="1:49">
+      <c r="A67" s="8"/>
+      <c r="B67" s="7"/>
       <c r="C67" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G67" s="3"/>
       <c r="H67" s="3"/>
@@ -5720,20 +6043,20 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2"/>
-      <c r="B68" s="3"/>
+    <row r="68" spans="1:49">
+      <c r="A68" s="8"/>
+      <c r="B68" s="7"/>
       <c r="C68" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G68" s="3"/>
       <c r="H68" s="3"/>
@@ -5783,20 +6106,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2"/>
-      <c r="B69" s="3"/>
+    <row r="69" spans="1:49">
+      <c r="A69" s="8"/>
+      <c r="B69" s="7"/>
       <c r="C69" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G69" s="3">
         <v>2</v>
@@ -5848,20 +6171,20 @@
         <v>23</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="2"/>
-      <c r="B70" s="3"/>
+    <row r="70" spans="1:49">
+      <c r="A70" s="8"/>
+      <c r="B70" s="7"/>
       <c r="C70" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G70" s="3"/>
       <c r="H70" s="3"/>
@@ -5911,20 +6234,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="2"/>
-      <c r="B71" s="3"/>
+    <row r="71" spans="1:49">
+      <c r="A71" s="8"/>
+      <c r="B71" s="7"/>
       <c r="C71" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G71" s="3">
         <v>1</v>
@@ -5974,24 +6297,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:49">
       <c r="A72" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
@@ -6045,24 +6368,24 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B73" s="2" t="s">
+    <row r="73" spans="1:49">
+      <c r="A73" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>221</v>
+      <c r="B73" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="F73" s="8" t="s">
+        <v>220</v>
       </c>
       <c r="G73" s="3">
         <v>37</v>
@@ -6148,16 +6471,17 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="R1:T1"/>
+    <mergeCell ref="W1:X1"/>
+    <mergeCell ref="Y1:AA1"/>
+    <mergeCell ref="AE1:AO1"/>
+    <mergeCell ref="AW1:AW2"/>
     <mergeCell ref="B12:B71"/>
     <mergeCell ref="A12:A71"/>
     <mergeCell ref="A73:F73"/>
     <mergeCell ref="J1:L1"/>
     <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="R1:T1"/>
-    <mergeCell ref="W1:X1"/>
-    <mergeCell ref="Y1:AA1"/>
-    <mergeCell ref="AE1:AO1"/>
-    <mergeCell ref="AW1:AW2"/>
   </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>